<commit_message>
updated pinout table prepared schematics
</commit_message>
<xml_diff>
--- a/serial_parallel_interface.xlsx
+++ b/serial_parallel_interface.xlsx
@@ -5,16 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian\Documents\Uni\Master\WISE2122\EALProjektpraktikum\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian\Documents\Uni\Master\WISE2122\EALProjektpraktikum\uz_d_encoder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2DE9088-A5B8-47E0-BF69-0C06552BEBF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC20B02A-273E-4E1F-B687-88E5859FA30D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10996" activeTab="1" xr2:uid="{19E285B5-7740-4A15-AD9F-8C8F45469901}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10996" activeTab="3" xr2:uid="{19E285B5-7740-4A15-AD9F-8C8F45469901}"/>
   </bookViews>
   <sheets>
     <sheet name="Signals" sheetId="1" r:id="rId1"/>
     <sheet name="Pinout" sheetId="2" r:id="rId2"/>
+    <sheet name="Tabelle1" sheetId="3" r:id="rId3"/>
+    <sheet name="Tabelle2" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="146">
   <si>
     <t>DIR</t>
   </si>
@@ -428,13 +430,58 @@
   </si>
   <si>
     <t>SELECTABLE</t>
+  </si>
+  <si>
+    <t>Resistor on board required or dip switch</t>
+  </si>
+  <si>
+    <t>Incremental</t>
+  </si>
+  <si>
+    <t>Resolver Parallel</t>
+  </si>
+  <si>
+    <t>Place Pull up!</t>
+  </si>
+  <si>
+    <t>Resolver Required</t>
+  </si>
+  <si>
+    <t>Resolver Incremental</t>
+  </si>
+  <si>
+    <t>Serial Resolver</t>
+  </si>
+  <si>
+    <t>Inc A</t>
+  </si>
+  <si>
+    <t>Inc B</t>
+  </si>
+  <si>
+    <t>Parallel Resolver</t>
+  </si>
+  <si>
+    <t>Analog</t>
+  </si>
+  <si>
+    <t>Absolute</t>
+  </si>
+  <si>
+    <t>Incremental Resolver</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>Parallel Nutzbar</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -456,8 +503,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -488,8 +548,38 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -497,21 +587,51 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1150,7 +1270,9 @@
       <c r="E19" t="s">
         <v>37</v>
       </c>
-      <c r="F19" s="2"/>
+      <c r="F19" s="2" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
@@ -1304,7 +1426,9 @@
       <c r="B30" t="s">
         <v>40</v>
       </c>
-      <c r="C30" s="3"/>
+      <c r="C30" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="D30" t="s">
         <v>36</v>
       </c>
@@ -1326,7 +1450,9 @@
       <c r="B31" t="s">
         <v>40</v>
       </c>
-      <c r="C31" s="3"/>
+      <c r="C31" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="D31" t="s">
         <v>36</v>
       </c>
@@ -1341,7 +1467,9 @@
       <c r="B32" t="s">
         <v>41</v>
       </c>
-      <c r="C32" s="3"/>
+      <c r="C32" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="D32" t="s">
         <v>37</v>
       </c>
@@ -1352,14 +1480,16 @@
         <v>38</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>2</v>
       </c>
       <c r="B33" t="s">
         <v>41</v>
       </c>
-      <c r="C33" s="3"/>
+      <c r="C33" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="D33" t="s">
         <v>37</v>
       </c>
@@ -1370,14 +1500,16 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>21</v>
       </c>
       <c r="B35" t="s">
         <v>40</v>
       </c>
-      <c r="C35" s="3"/>
+      <c r="C35" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="D35" t="s">
         <v>35</v>
       </c>
@@ -1387,15 +1519,20 @@
       <c r="F35" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G35" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>8</v>
       </c>
       <c r="B36" t="s">
         <v>40</v>
       </c>
-      <c r="C36" s="3"/>
+      <c r="C36" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="D36" t="s">
         <v>35</v>
       </c>
@@ -1405,23 +1542,31 @@
       <c r="F36" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G36" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>11</v>
       </c>
       <c r="B37" t="s">
         <v>40</v>
       </c>
-      <c r="C37" s="3"/>
+      <c r="C37" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="D37" t="s">
         <v>43</v>
       </c>
       <c r="E37" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G37" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>47</v>
       </c>
@@ -1431,15 +1576,15 @@
       </c>
       <c r="C39">
         <f>COUNTIF(C3:C37, "connected")</f>
-        <v>21</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.45">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A41" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>50</v>
       </c>
@@ -1447,7 +1592,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>51</v>
       </c>
@@ -1455,7 +1600,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>52</v>
       </c>
@@ -1463,7 +1608,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>53</v>
       </c>
@@ -1471,7 +1616,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>54</v>
       </c>
@@ -1479,7 +1624,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>55</v>
       </c>
@@ -1648,10 +1793,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="6"/>
+      <c r="C1" s="20"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
@@ -1665,7 +1810,7 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>79</v>
       </c>
       <c r="B3" t="s">
@@ -1673,7 +1818,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>78</v>
       </c>
       <c r="B4" t="s">
@@ -1681,7 +1826,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>80</v>
       </c>
       <c r="B5" t="s">
@@ -1689,7 +1834,7 @@
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>81</v>
       </c>
       <c r="B6" t="s">
@@ -1697,7 +1842,7 @@
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="6" t="s">
         <v>82</v>
       </c>
       <c r="B7" t="s">
@@ -1705,7 +1850,7 @@
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="6" t="s">
         <v>77</v>
       </c>
       <c r="B8" t="s">
@@ -1866,7 +2011,7 @@
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="6" t="s">
         <v>99</v>
       </c>
       <c r="B27" t="s">
@@ -1874,7 +2019,7 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="6" t="s">
         <v>100</v>
       </c>
       <c r="B28" t="s">
@@ -1882,7 +2027,7 @@
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A29" s="7" t="s">
+      <c r="A29" s="6" t="s">
         <v>101</v>
       </c>
       <c r="B29" t="s">
@@ -1890,7 +2035,7 @@
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A30" s="7" t="s">
+      <c r="A30" s="6" t="s">
         <v>102</v>
       </c>
       <c r="B30" t="s">
@@ -1898,7 +2043,7 @@
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A31" s="7" t="s">
+      <c r="A31" s="6" t="s">
         <v>103</v>
       </c>
       <c r="B31" t="s">
@@ -1906,7 +2051,7 @@
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A32" s="7" t="s">
+      <c r="A32" s="6" t="s">
         <v>104</v>
       </c>
       <c r="B32" t="s">
@@ -1920,4 +2065,1171 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A2FD9E5-FD85-4AC4-A77E-D9AF5188DE92}">
+  <dimension ref="A1:M31"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="4" max="4" width="20.9296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="8" width="17.86328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.53125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A2" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A3" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A4" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A5" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A6" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A7" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>86</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>87</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>89</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F16" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="G16" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="J16" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="K16" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="L16" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="M16" s="14" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="G17" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="H17" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="I17" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="16"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="F18" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="G18" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="H18" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="I18" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="16"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="F19" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="G19" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="H19" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="I19" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="16"/>
+      <c r="M19" s="16"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="F20" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="K20" s="16"/>
+      <c r="L20" s="16"/>
+      <c r="M20" s="16"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="G21" s="16"/>
+      <c r="H21" s="16"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="L21" s="16"/>
+      <c r="M21" s="16"/>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>95</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F22" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="G22" s="16"/>
+      <c r="H22" s="16"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="M22" s="16"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>96</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="G23" s="16"/>
+      <c r="H23" s="16"/>
+      <c r="I23" s="16"/>
+      <c r="J23" s="16"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="16"/>
+      <c r="M23" s="15" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>97</v>
+      </c>
+      <c r="B24" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>98</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A26" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A27" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A28" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A29" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A30" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A31" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71BA19D0-A05D-43AE-B8FD-7DE6E3441DDE}">
+  <dimension ref="A1:T38"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="1" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A2" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A3" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A4" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A5" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A6" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A7" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="L11" s="17"/>
+      <c r="M11" s="17"/>
+      <c r="T11" s="11" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="L12" s="17"/>
+      <c r="M12" s="17"/>
+      <c r="T12" s="10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>86</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="T13" s="3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>87</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="T14" s="7" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="T15" s="8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>89</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="T16" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>95</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>96</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>97</v>
+      </c>
+      <c r="B24" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" t="s">
+        <v>72</v>
+      </c>
+      <c r="D24" t="s">
+        <v>72</v>
+      </c>
+      <c r="E24" t="s">
+        <v>72</v>
+      </c>
+      <c r="F24" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>98</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A26" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A27" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A28" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D28" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A29" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D29" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A30" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A31" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A33" s="18"/>
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="12"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A34" s="18"/>
+      <c r="B34" s="19"/>
+      <c r="C34" s="19"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="19"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A35" s="18"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A36" s="18"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A37" s="18"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="B38" s="20"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B38:D38"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
most of the hardware changes (schematic) finished, i2c port expander missing
</commit_message>
<xml_diff>
--- a/serial_parallel_interface.xlsx
+++ b/serial_parallel_interface.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian\Documents\Uni\Master\WISE2122\EALProjektpraktikum\uz_d_encoder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC20B02A-273E-4E1F-B687-88E5859FA30D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{935FE062-F200-4987-95B3-2C698D724E7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10996" activeTab="3" xr2:uid="{19E285B5-7740-4A15-AD9F-8C8F45469901}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="4" xr2:uid="{19E285B5-7740-4A15-AD9F-8C8F45469901}"/>
   </bookViews>
   <sheets>
     <sheet name="Signals" sheetId="1" r:id="rId1"/>
-    <sheet name="Pinout" sheetId="2" r:id="rId2"/>
-    <sheet name="Tabelle1" sheetId="3" r:id="rId3"/>
-    <sheet name="Tabelle2" sheetId="4" r:id="rId4"/>
+    <sheet name="Tabelle3" sheetId="5" r:id="rId2"/>
+    <sheet name="Pinout" sheetId="2" r:id="rId3"/>
+    <sheet name="Tabelle1" sheetId="3" r:id="rId4"/>
+    <sheet name="Tabelle2" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="705" uniqueCount="181">
   <si>
     <t>DIR</t>
   </si>
@@ -420,9 +421,6 @@
     <t>RESOLVER_NM</t>
   </si>
   <si>
-    <t>Not connected</t>
-  </si>
-  <si>
     <t>NOT REQ</t>
   </si>
   <si>
@@ -475,6 +473,114 @@
   </si>
   <si>
     <t>Parallel Nutzbar</t>
+  </si>
+  <si>
+    <t>1B3</t>
+  </si>
+  <si>
+    <t>2B3</t>
+  </si>
+  <si>
+    <t>3B3</t>
+  </si>
+  <si>
+    <t>S0</t>
+  </si>
+  <si>
+    <t>GND</t>
+  </si>
+  <si>
+    <t>VCC</t>
+  </si>
+  <si>
+    <t>1A</t>
+  </si>
+  <si>
+    <t>2A</t>
+  </si>
+  <si>
+    <t>3A</t>
+  </si>
+  <si>
+    <t>4A</t>
+  </si>
+  <si>
+    <t>4B3</t>
+  </si>
+  <si>
+    <t>5A</t>
+  </si>
+  <si>
+    <t>5B3</t>
+  </si>
+  <si>
+    <t>6A</t>
+  </si>
+  <si>
+    <t>7A</t>
+  </si>
+  <si>
+    <t>7B3</t>
+  </si>
+  <si>
+    <t>8A</t>
+  </si>
+  <si>
+    <t>8B3</t>
+  </si>
+  <si>
+    <t>9A</t>
+  </si>
+  <si>
+    <t>9B3</t>
+  </si>
+  <si>
+    <t>10A</t>
+  </si>
+  <si>
+    <t>10B3</t>
+  </si>
+  <si>
+    <t>11A</t>
+  </si>
+  <si>
+    <t>11B3</t>
+  </si>
+  <si>
+    <t>12A</t>
+  </si>
+  <si>
+    <t>12B3</t>
+  </si>
+  <si>
+    <t>DIG_IO_0</t>
+  </si>
+  <si>
+    <t>DIG_IO_1</t>
+  </si>
+  <si>
+    <t>DIG_IO_2</t>
+  </si>
+  <si>
+    <t>DIG_IO_3</t>
+  </si>
+  <si>
+    <t>DIG_IO_4</t>
+  </si>
+  <si>
+    <t>DIG_IO_5</t>
+  </si>
+  <si>
+    <t>DIG_IO_6</t>
+  </si>
+  <si>
+    <t>DIG_IO_7</t>
+  </si>
+  <si>
+    <t>DIG_IO_8</t>
+  </si>
+  <si>
+    <t>DIG_IO_9</t>
   </si>
 </sst>
 </file>
@@ -947,18 +1053,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4CB6542-F889-4043-9BB2-4053567E6D12}">
   <dimension ref="A1:M72"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.6640625" customWidth="1"/>
-    <col min="4" max="4" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.06640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.06640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" customWidth="1"/>
+    <col min="4" max="4" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
@@ -975,14 +1081,14 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>48</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -999,7 +1105,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -1016,7 +1122,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -1033,7 +1139,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -1050,7 +1156,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -1067,7 +1173,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>23</v>
       </c>
@@ -1084,7 +1190,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1101,7 +1207,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -1118,7 +1224,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1135,7 +1241,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -1152,7 +1258,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -1169,7 +1275,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>29</v>
       </c>
@@ -1186,7 +1292,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -1203,7 +1309,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -1222,7 +1328,7 @@
       <c r="F16" s="2"/>
       <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -1239,7 +1345,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -1256,7 +1362,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>9</v>
       </c>
@@ -1271,10 +1377,10 @@
         <v>37</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>1</v>
       </c>
@@ -1285,7 +1391,7 @@
         <v>41</v>
       </c>
       <c r="D21" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E21" t="s">
         <v>37</v>
@@ -1294,7 +1400,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>10</v>
       </c>
@@ -1314,7 +1420,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>12</v>
       </c>
@@ -1331,7 +1437,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>4</v>
       </c>
@@ -1342,13 +1448,13 @@
         <v>70</v>
       </c>
       <c r="D25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E25" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>5</v>
       </c>
@@ -1359,13 +1465,13 @@
         <v>70</v>
       </c>
       <c r="D26" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E26" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>17</v>
       </c>
@@ -1376,13 +1482,13 @@
         <v>70</v>
       </c>
       <c r="D27" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E27" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>0</v>
       </c>
@@ -1393,13 +1499,13 @@
         <v>41</v>
       </c>
       <c r="D28" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E28" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>18</v>
       </c>
@@ -1416,10 +1522,10 @@
         <v>36</v>
       </c>
       <c r="F29" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>19</v>
       </c>
@@ -1443,7 +1549,7 @@
       <c r="L30" s="5"/>
       <c r="M30" s="5"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>20</v>
       </c>
@@ -1460,7 +1566,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>3</v>
       </c>
@@ -1480,7 +1586,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -1500,7 +1606,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>21</v>
       </c>
@@ -1520,10 +1626,10 @@
         <v>38</v>
       </c>
       <c r="G35" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -1543,10 +1649,10 @@
         <v>38</v>
       </c>
       <c r="G36" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>11</v>
       </c>
@@ -1563,10 +1669,10 @@
         <v>44</v>
       </c>
       <c r="G37" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>47</v>
       </c>
@@ -1579,12 +1685,12 @@
         <v>23</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>50</v>
       </c>
@@ -1592,7 +1698,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>51</v>
       </c>
@@ -1600,7 +1706,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>52</v>
       </c>
@@ -1608,7 +1714,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>53</v>
       </c>
@@ -1616,7 +1722,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>54</v>
       </c>
@@ -1624,7 +1730,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>55</v>
       </c>
@@ -1632,12 +1738,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>56</v>
       </c>
@@ -1645,7 +1751,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>57</v>
       </c>
@@ -1653,7 +1759,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>58</v>
       </c>
@@ -1661,12 +1767,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>59</v>
       </c>
@@ -1674,7 +1780,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>60</v>
       </c>
@@ -1682,7 +1788,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>61</v>
       </c>
@@ -1690,12 +1796,12 @@
         <v>70</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>64</v>
       </c>
@@ -1703,7 +1809,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>65</v>
       </c>
@@ -1711,7 +1817,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>66</v>
       </c>
@@ -1719,7 +1825,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>67</v>
       </c>
@@ -1727,7 +1833,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>68</v>
       </c>
@@ -1735,7 +1841,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>69</v>
       </c>
@@ -1743,7 +1849,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>72</v>
       </c>
@@ -1751,7 +1857,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>47</v>
       </c>
@@ -1760,7 +1866,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>74</v>
       </c>
@@ -1769,7 +1875,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>73</v>
       </c>
@@ -1785,20 +1891,339 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{886C181C-1C4F-445C-BC6A-0C497DE68EAB}">
+  <dimension ref="A1:B46"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="3"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>0</v>
+      </c>
+      <c r="B24" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B25" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>2</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>72</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B80DC29B-7AAE-432E-95FD-36A6EDE8D593}">
   <dimension ref="A1:C32"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.73046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B1" s="20" t="s">
         <v>39</v>
       </c>
       <c r="C1" s="20"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>105</v>
       </c>
@@ -1809,7 +2234,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>79</v>
       </c>
@@ -1817,7 +2242,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>78</v>
       </c>
@@ -1825,7 +2250,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>80</v>
       </c>
@@ -1833,7 +2258,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>81</v>
       </c>
@@ -1841,7 +2266,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>82</v>
       </c>
@@ -1849,7 +2274,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>77</v>
       </c>
@@ -1857,7 +2282,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>76</v>
       </c>
@@ -1865,7 +2290,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>75</v>
       </c>
@@ -1873,7 +2298,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>83</v>
       </c>
@@ -1881,7 +2306,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>84</v>
       </c>
@@ -1889,7 +2314,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>85</v>
       </c>
@@ -1897,7 +2322,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>86</v>
       </c>
@@ -1905,7 +2330,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>87</v>
       </c>
@@ -1913,7 +2338,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>88</v>
       </c>
@@ -1921,7 +2346,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>89</v>
       </c>
@@ -1932,7 +2357,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>90</v>
       </c>
@@ -1943,7 +2368,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>91</v>
       </c>
@@ -1954,7 +2379,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>92</v>
       </c>
@@ -1962,7 +2387,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>93</v>
       </c>
@@ -1970,7 +2395,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>94</v>
       </c>
@@ -1978,7 +2403,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>95</v>
       </c>
@@ -1986,7 +2411,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>96</v>
       </c>
@@ -1994,7 +2419,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>97</v>
       </c>
@@ -2002,7 +2427,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>98</v>
       </c>
@@ -2010,7 +2435,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>99</v>
       </c>
@@ -2018,7 +2443,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>100</v>
       </c>
@@ -2026,7 +2451,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>101</v>
       </c>
@@ -2034,7 +2459,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>102</v>
       </c>
@@ -2042,7 +2467,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>103</v>
       </c>
@@ -2050,12 +2475,12 @@
         <v>123</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>104</v>
       </c>
       <c r="B32" t="s">
-        <v>127</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -2067,22 +2492,22 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A2FD9E5-FD85-4AC4-A77E-D9AF5188DE92}">
   <dimension ref="A1:M31"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="20.9296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="8" width="17.86328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.53125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="8" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>79</v>
       </c>
@@ -2093,7 +2518,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>78</v>
       </c>
@@ -2104,7 +2529,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>80</v>
       </c>
@@ -2115,7 +2540,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>81</v>
       </c>
@@ -2126,10 +2551,10 @@
         <v>67</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>82</v>
       </c>
@@ -2140,10 +2565,10 @@
         <v>68</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>77</v>
       </c>
@@ -2154,10 +2579,10 @@
         <v>69</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>76</v>
       </c>
@@ -2168,10 +2593,10 @@
         <v>4</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>75</v>
       </c>
@@ -2185,7 +2610,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>83</v>
       </c>
@@ -2199,7 +2624,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>84</v>
       </c>
@@ -2210,7 +2635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>85</v>
       </c>
@@ -2224,7 +2649,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>86</v>
       </c>
@@ -2238,7 +2663,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>87</v>
       </c>
@@ -2252,7 +2677,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>88</v>
       </c>
@@ -2266,7 +2691,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>89</v>
       </c>
@@ -2280,31 +2705,31 @@
         <v>68</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H16" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="J16" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="K16" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="L16" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="I16" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="J16" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="K16" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="L16" s="14" t="s">
+      <c r="M16" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="M16" s="14" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>90</v>
       </c>
@@ -2318,23 +2743,23 @@
         <v>69</v>
       </c>
       <c r="F17" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="G17" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="G17" s="15" t="s">
-        <v>144</v>
-      </c>
       <c r="H17" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J17" s="16"/>
       <c r="K17" s="16"/>
       <c r="L17" s="16"/>
       <c r="M17" s="16"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>91</v>
       </c>
@@ -2348,23 +2773,23 @@
         <v>50</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G18" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I18" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J18" s="16"/>
       <c r="K18" s="16"/>
       <c r="L18" s="16"/>
       <c r="M18" s="16"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>92</v>
       </c>
@@ -2378,23 +2803,23 @@
         <v>51</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G19" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H19" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I19" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J19" s="16"/>
       <c r="K19" s="16"/>
       <c r="L19" s="16"/>
       <c r="M19" s="16"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>93</v>
       </c>
@@ -2408,19 +2833,19 @@
         <v>52</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
       <c r="I20" s="16"/>
       <c r="J20" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="K20" s="16"/>
       <c r="L20" s="16"/>
       <c r="M20" s="16"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>94</v>
       </c>
@@ -2434,19 +2859,19 @@
         <v>53</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
       <c r="I21" s="16"/>
       <c r="J21" s="16"/>
       <c r="K21" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="L21" s="16"/>
       <c r="M21" s="16"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>95</v>
       </c>
@@ -2460,7 +2885,7 @@
         <v>54</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="16"/>
@@ -2468,11 +2893,11 @@
       <c r="J22" s="16"/>
       <c r="K22" s="16"/>
       <c r="L22" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="M22" s="16"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>96</v>
       </c>
@@ -2486,7 +2911,7 @@
         <v>55</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
@@ -2495,10 +2920,10 @@
       <c r="K23" s="16"/>
       <c r="L23" s="16"/>
       <c r="M23" s="15" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>97</v>
       </c>
@@ -2506,7 +2931,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>98</v>
       </c>
@@ -2514,7 +2939,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>99</v>
       </c>
@@ -2525,7 +2950,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>100</v>
       </c>
@@ -2536,7 +2961,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>101</v>
       </c>
@@ -2547,7 +2972,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>102</v>
       </c>
@@ -2558,7 +2983,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>103</v>
       </c>
@@ -2569,7 +2994,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>104</v>
       </c>
@@ -2586,17 +3011,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71BA19D0-A05D-43AE-B8FD-7DE6E3441DDE}">
-  <dimension ref="A1:T38"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:T44"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="22.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>79</v>
       </c>
@@ -2616,7 +3044,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>78</v>
       </c>
@@ -2636,7 +3064,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>80</v>
       </c>
@@ -2656,7 +3084,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>81</v>
       </c>
@@ -2676,7 +3104,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>82</v>
       </c>
@@ -2696,7 +3124,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>77</v>
       </c>
@@ -2716,7 +3144,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>76</v>
       </c>
@@ -2730,7 +3158,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>75</v>
       </c>
@@ -2747,7 +3175,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>83</v>
       </c>
@@ -2764,7 +3192,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>84</v>
       </c>
@@ -2784,12 +3212,14 @@
       <c r="H11" s="17"/>
       <c r="I11" s="17"/>
       <c r="L11" s="17"/>
-      <c r="M11" s="17"/>
+      <c r="M11" s="17" t="s">
+        <v>171</v>
+      </c>
       <c r="T11" s="11" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.45">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>85</v>
       </c>
@@ -2809,12 +3239,14 @@
       <c r="H12" s="17"/>
       <c r="I12" s="17"/>
       <c r="L12" s="17"/>
-      <c r="M12" s="17"/>
+      <c r="M12" s="17" t="s">
+        <v>172</v>
+      </c>
       <c r="T12" s="10" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.45">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>86</v>
       </c>
@@ -2830,11 +3262,14 @@
       <c r="F13" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="M13" s="17" t="s">
+        <v>173</v>
+      </c>
       <c r="T13" s="3" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.45">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>87</v>
       </c>
@@ -2853,11 +3288,14 @@
       <c r="F14" s="3" t="s">
         <v>12</v>
       </c>
+      <c r="M14" s="17" t="s">
+        <v>174</v>
+      </c>
       <c r="T14" s="7" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.45">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>88</v>
       </c>
@@ -2876,11 +3314,14 @@
       <c r="F15" s="3" t="s">
         <v>18</v>
       </c>
+      <c r="M15" s="17" t="s">
+        <v>175</v>
+      </c>
       <c r="T15" s="8" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>89</v>
       </c>
@@ -2899,11 +3340,14 @@
       <c r="F16" s="3" t="s">
         <v>3</v>
       </c>
+      <c r="M16" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="T16" s="9" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>90</v>
       </c>
@@ -2922,8 +3366,14 @@
       <c r="F17" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="K17" t="s">
+        <v>148</v>
+      </c>
+      <c r="M17" s="17" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>91</v>
       </c>
@@ -2942,8 +3392,14 @@
       <c r="F18" s="7" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="K18" t="s">
+        <v>151</v>
+      </c>
+      <c r="M18" s="17" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>92</v>
       </c>
@@ -2962,8 +3418,14 @@
       <c r="F19" s="7" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="K19" t="s">
+        <v>145</v>
+      </c>
+      <c r="M19" s="17" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>93</v>
       </c>
@@ -2982,8 +3444,14 @@
       <c r="F20" s="7" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="K20" t="s">
+        <v>152</v>
+      </c>
+      <c r="M20" s="17" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>94</v>
       </c>
@@ -3002,8 +3470,11 @@
       <c r="F21" s="7" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="K21" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>95</v>
       </c>
@@ -3022,8 +3493,11 @@
       <c r="F22" s="7" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="K22" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>96</v>
       </c>
@@ -3042,8 +3516,11 @@
       <c r="F23" s="7" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="K23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>97</v>
       </c>
@@ -3062,8 +3539,11 @@
       <c r="F24" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="K24" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>98</v>
       </c>
@@ -3076,8 +3556,11 @@
       <c r="D25" s="10" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="K25" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>99</v>
       </c>
@@ -3096,8 +3579,11 @@
       <c r="F26" s="9" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="K26" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>100</v>
       </c>
@@ -3116,8 +3602,11 @@
       <c r="F27" s="9" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="K27" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>101</v>
       </c>
@@ -3136,48 +3625,34 @@
       <c r="F28" s="9" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A29" s="6" t="s">
+      <c r="K28" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B30" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C30" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D30" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="E29" s="9" t="s">
+      <c r="E30" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F29" s="9" t="s">
+      <c r="F30" s="9" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A30" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="B30" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="C30" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="D30" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="E30" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F30" s="9" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="K30" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>104</v>
       </c>
@@ -3196,40 +3671,97 @@
       <c r="F31" s="9" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="K31" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K32" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="18"/>
       <c r="B33" s="20"/>
       <c r="C33" s="20"/>
       <c r="D33" s="20"/>
       <c r="E33" s="12"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="K33" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="18"/>
       <c r="B34" s="19"/>
       <c r="C34" s="19"/>
       <c r="D34" s="19"/>
       <c r="E34" s="19"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="K34" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="18"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="K35" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="18"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="K36" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="18"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="K37" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B38" s="20"/>
       <c r="C38" s="20"/>
       <c r="D38" s="20"/>
+      <c r="K38" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K39" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K40" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K41" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K42" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K43" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K44" t="s">
+        <v>170</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="B38:D38"/>
   </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>